<commit_message>
Update application and Supabase integration
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -413,7 +413,7 @@
         <v>Route Count</v>
       </c>
       <c r="B2">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -425,7 +425,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -572,7 +572,7 @@
         <v>EP-007</v>
       </c>
       <c r="B8" t="str">
-        <v>/history</v>
+        <v>/forgot-password</v>
       </c>
       <c r="C8" t="str">
         <v>GET</v>
@@ -592,7 +592,7 @@
         <v>EP-008</v>
       </c>
       <c r="B9" t="str">
-        <v>/login</v>
+        <v>/history</v>
       </c>
       <c r="C9" t="str">
         <v>GET</v>
@@ -612,7 +612,7 @@
         <v>EP-009</v>
       </c>
       <c r="B10" t="str">
-        <v>/profile</v>
+        <v>/login</v>
       </c>
       <c r="C10" t="str">
         <v>GET</v>
@@ -632,7 +632,7 @@
         <v>EP-010</v>
       </c>
       <c r="B11" t="str">
-        <v>/register</v>
+        <v>/profile</v>
       </c>
       <c r="C11" t="str">
         <v>GET</v>
@@ -652,7 +652,7 @@
         <v>EP-011</v>
       </c>
       <c r="B12" t="str">
-        <v>/send-sos</v>
+        <v>/register</v>
       </c>
       <c r="C12" t="str">
         <v>GET</v>
@@ -672,7 +672,7 @@
         <v>EP-012</v>
       </c>
       <c r="B13" t="str">
-        <v>/settings</v>
+        <v>/reset-password</v>
       </c>
       <c r="C13" t="str">
         <v>GET</v>
@@ -692,7 +692,7 @@
         <v>EP-013</v>
       </c>
       <c r="B14" t="str">
-        <v>/tracking</v>
+        <v>/send-sos</v>
       </c>
       <c r="C14" t="str">
         <v>GET</v>
@@ -712,24 +712,104 @@
         <v>EP-014</v>
       </c>
       <c r="B15" t="str">
+        <v>/settings</v>
+      </c>
+      <c r="C15" t="str">
+        <v>GET</v>
+      </c>
+      <c r="D15" t="str">
+        <v>UI route available in the application</v>
+      </c>
+      <c r="E15" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Protected or public application route</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>EP-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>/tracking</v>
+      </c>
+      <c r="C16" t="str">
+        <v>GET</v>
+      </c>
+      <c r="D16" t="str">
+        <v>UI route available in the application</v>
+      </c>
+      <c r="E16" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Protected or public application route</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>EP-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>/verify-email</v>
+      </c>
+      <c r="C17" t="str">
+        <v>GET</v>
+      </c>
+      <c r="D17" t="str">
+        <v>UI route available in the application</v>
+      </c>
+      <c r="E17" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Protected or public application route</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>EP-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>/verify-email-pending</v>
+      </c>
+      <c r="C18" t="str">
+        <v>GET</v>
+      </c>
+      <c r="D18" t="str">
+        <v>UI route available in the application</v>
+      </c>
+      <c r="E18" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Protected or public application route</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>EP-018</v>
+      </c>
+      <c r="B19" t="str">
         <v>/volunteer</v>
       </c>
-      <c r="C15" t="str">
-        <v>GET</v>
-      </c>
-      <c r="D15" t="str">
-        <v>UI route available in the application</v>
-      </c>
-      <c r="E15" t="str">
-        <v>src/App.tsx</v>
-      </c>
-      <c r="F15" t="str">
+      <c r="C19" t="str">
+        <v>GET</v>
+      </c>
+      <c r="D19" t="str">
+        <v>UI route available in the application</v>
+      </c>
+      <c r="E19" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="F19" t="str">
         <v>Protected or public application route</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>